<commit_message>
Etapa 9: first real cost input and its margin consequences
Founder benchmark: a good passive-service SDR costs R$6,000/month.
Converted to productive-hour cost (132h/month): R$47.73 under PJ,
R$79.55 under CLT with charges. Modeled both: the typical client is
highly profitable either way (74% and 62% contribution margin), but the
P90 tail flips to a R$56/month loss under CLT - which reclassifies the
beta limits from measurement instrument to mandatory margin protection,
given the interviews signalled universal usage. Records the caveat that
a passive SDR is below the seniority the operation actually needs, so
the CLT case may be the optimistic one, and elevates the hiring regime
to a margin decision for Etapa 15. Spreadsheet defaults updated with
the real figures.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143F1DWyj4AQrbnXjF2cgaY
</commit_message>
<xml_diff>
--- a/deixa-comigo/financeiro/Deixa_Comigo_Unit_Economics.xlsx
+++ b/deixa-comigo/financeiro/Deixa_Comigo_Unit_Economics.xlsx
@@ -168,9 +168,9 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="C8" s="6">
-        <f>-'Premissas'!C14*'Custo da Missão'!C18</f>
+        <f>-'Premissas'!C16*'Custo da Missão'!C18</f>
         <v/>
       </c>
     </row>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>'Premissas'!C18</f>
+        <f>'Premissas'!C20</f>
         <v/>
       </c>
     </row>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="C15" s="6">
-        <f>C6-'Custo da Missão'!C21-'Premissas'!C14*'Custo da Missão'!C19</f>
+        <f>C6-'Custo da Missão'!C21-'Premissas'!C16*'Custo da Missão'!C19</f>
         <v/>
       </c>
     </row>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="C20" s="13">
-        <f>'Premissas'!C20</f>
+        <f>'Premissas'!C22</f>
         <v/>
       </c>
     </row>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="C30" s="18">
-        <f>IF('Premissas'!C19=0,0,ROUNDUP(C28/'Premissas'!C19,1))</f>
+        <f>IF('Premissas'!C21=0,0,ROUNDUP(C28/'Premissas'!C21,1))</f>
         <v/>
       </c>
     </row>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="C34" s="15">
-        <f>'Premissas'!C23</f>
+        <f>'Premissas'!C25</f>
         <v/>
       </c>
     </row>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="C36" s="15">
-        <f>'Premissas'!C24</f>
+        <f>'Premissas'!C26</f>
         <v/>
       </c>
     </row>
@@ -911,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E24"/>
+  <dimension ref="B1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1024,143 +1024,173 @@
         </is>
       </c>
       <c r="C12" s="19" t="n">
-        <v>50</v>
+        <v>79.55</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>⚠ PEDIR AO FORNECEDOR (porta 15.1). Inclui encargos, gestão e ociosidade.</t>
+          <t>Fundador 31/07: SDR bom = R$ 6.000/mês. CLT c/ encargos (x1,75) = R$ 10.500 / 132h = R$ 79,55. Se PJ: use 47,73.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Custo/hora de especialista (escalonamento)</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="n">
-        <v>120</v>
+          <t xml:space="preserve">  [ref] Salário mensal do operador</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>6000</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Casos que sobem para profissional habilitado.</t>
+          <t>Fonte: fundador, 31/07/2026 — SDR de atendimento passivo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Custo de IA/software por missão</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>3</v>
+          <t xml:space="preserve">  [ref] Multiplicador de encargos</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>1.75</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Tokens, telefonia, integrações.</t>
+          <t>CLT ~1,75 · PJ ~1,05. Célula de referência: recalcule a linha 12 se mudar.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>Custo/hora de especialista (escalonamento)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>120</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Casos que sobem para profissional habilitado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Custo de IA/software por missão</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Tokens, telefonia, integrações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
           <t>% das missões que escalam para especialista</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C17" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Medir no piloto.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>METAS E CENÁRIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Margem-alvo mínima (porta 9.4)</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Trava do motor: abaixo disso a conta não fecha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Horas produtivas por operador/mês</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="n">
-        <v>132</v>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Ex.: 176h contratuais × 75% de produtividade.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Margem-alvo mínima (porta 9.4)</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Trava do motor: abaixo disso a conta não fecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Horas produtivas por operador/mês</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>132</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Ex.: 176h contratuais × 75% de produtividade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t>Nº de pessoas cuidadas no cenário</t>
         </is>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C22" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Objetivo da Etapa 6: 300 até jul/2027.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>CONTEXTO SOCIETÁRIO (para o alerta do Simples)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Receita anual das outras empresas do sócio</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n">
+      <c r="C25" s="21" t="n">
         <v>4200000</v>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Setfree: R$ 350k/mês x 12. Fonte: fundador, 31/07/2026.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Teto da receita bruta global — Simples</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C26" s="21" t="n">
         <v>4800000</v>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>LC 123/2006. Confirmar vigência com a Cony Services.</t>
         </is>
@@ -1168,11 +1198,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B17:E17"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B19:E19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1237,13 +1267,13 @@
           <t>Agenda e acesso (marcar, remarcar, confirmar)</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="22" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -1253,13 +1283,13 @@
           <t>Documento claro (organizar e resumir)</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="22" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -1269,13 +1299,13 @@
           <t>Três opções prontas (comparar prestadores)</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>45</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1285,13 +1315,13 @@
           <t>Protocolo acompanhado (convênio, ouvidoria)</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1301,13 +1331,13 @@
           <t>Plano de próximos passos</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1317,13 +1347,13 @@
           <t>Família alinhada (atualização factual)</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>15</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1372,7 +1402,7 @@
         </is>
       </c>
       <c r="C17" s="6">
-        <f>C16/60*'Premissas'!C12+C16/60*'Premissas'!C15*('Premissas'!C13-'Premissas'!C12)</f>
+        <f>C16/60*'Premissas'!C12+C16/60*'Premissas'!C17*('Premissas'!C15-'Premissas'!C12)</f>
         <v/>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1496,7 +1526,7 @@
           <t>Coordenação / gestão da operação</t>
         </is>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="21" t="n">
         <v>8000</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1511,7 +1541,7 @@
           <t>Tecnologia base (WhatsApp API, hospedagem, banco)</t>
         </is>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="21" t="n">
         <v>1500</v>
       </c>
     </row>
@@ -1521,7 +1551,7 @@
           <t>Ferramentas e assinaturas</t>
         </is>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="21" t="n">
         <v>800</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1536,7 +1566,7 @@
           <t>Jurídico e contábil</t>
         </is>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="21" t="n">
         <v>2500</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1551,7 +1581,7 @@
           <t>Marketing e aquisição</t>
         </is>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="21" t="n">
         <v>5000</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1566,7 +1596,7 @@
           <t>Estrutura (endereço fiscal, banco, taxas)</t>
         </is>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="21" t="n">
         <v>700</v>
       </c>
     </row>
@@ -1576,7 +1606,7 @@
           <t>Outros / reserva</t>
         </is>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="21" t="n">
         <v>1500</v>
       </c>
     </row>
@@ -1604,7 +1634,7 @@
           <t>Caixa disponível hoje</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="21" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="inlineStr">

</xml_diff>